<commit_message>
Save JSON output to ../USD-LKR_Scraper directory
</commit_message>
<xml_diff>
--- a/WholeSale-Price-Model/data/raw/Amika.xlsx
+++ b/WholeSale-Price-Model/data/raw/Amika.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://liverguac-my.sharepoint.com/personal/a_siyambalapitiyage_rgu_ac_uk/Documents/Desktop/DSGP/DSGP_Group_38/WholeSale-Price-Model/data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="79" documentId="8_{DBDE29C9-DF6E-4BC9-ABC1-633918917E58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C5BB2C1E-A2BE-4000-906D-7C60AF14F936}"/>
+  <xr:revisionPtr revIDLastSave="83" documentId="8_{DBDE29C9-DF6E-4BC9-ABC1-633918917E58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1DBDB6B0-B88A-4BE7-919C-DECE394FEF83}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{215EF489-9573-4990-96B9-A28CAE1C2861}"/>
+    <workbookView xWindow="3552" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{215EF489-9573-4990-96B9-A28CAE1C2861}"/>
   </bookViews>
   <sheets>
     <sheet name="Wholesale" sheetId="2" r:id="rId1"/>
@@ -16983,9 +16983,7 @@
       <c r="K98" s="9">
         <v>235</v>
       </c>
-      <c r="L98" s="9">
-        <v>235</v>
-      </c>
+      <c r="L98" s="9"/>
       <c r="M98" s="8"/>
       <c r="N98" s="8"/>
       <c r="O98" s="8"/>
@@ -17063,10 +17061,8 @@
       <c r="K99" s="9">
         <v>105</v>
       </c>
-      <c r="L99" s="9">
-        <v>105</v>
-      </c>
-      <c r="M99" s="8"/>
+      <c r="L99" s="9"/>
+      <c r="M99" s="6"/>
       <c r="N99" s="8"/>
       <c r="O99" s="8"/>
       <c r="P99" s="8"/>
@@ -17143,9 +17139,7 @@
       <c r="K100" s="6">
         <v>125</v>
       </c>
-      <c r="L100" s="6">
-        <v>125</v>
-      </c>
+      <c r="L100" s="6"/>
       <c r="M100" s="6"/>
       <c r="N100" s="6"/>
       <c r="O100" s="6"/>
@@ -17223,9 +17217,7 @@
       <c r="K101" s="6">
         <v>135</v>
       </c>
-      <c r="L101" s="6">
-        <v>135</v>
-      </c>
+      <c r="L101" s="6"/>
       <c r="M101" s="6"/>
       <c r="N101" s="6"/>
       <c r="O101" s="6"/>
@@ -17303,9 +17295,7 @@
       <c r="K102" s="6">
         <v>105</v>
       </c>
-      <c r="L102" s="6">
-        <v>105</v>
-      </c>
+      <c r="L102" s="6"/>
       <c r="M102" s="6"/>
       <c r="N102" s="6"/>
       <c r="O102" s="6"/>
@@ -17383,9 +17373,7 @@
       <c r="K103" s="6">
         <v>290</v>
       </c>
-      <c r="L103" s="6">
-        <v>290</v>
-      </c>
+      <c r="L103" s="6"/>
       <c r="M103" s="6"/>
       <c r="N103" s="6"/>
       <c r="O103" s="6"/>

</xml_diff>

<commit_message>
changes in the backend
</commit_message>
<xml_diff>
--- a/WholeSale-Price-Model/data/raw/Amika.xlsx
+++ b/WholeSale-Price-Model/data/raw/Amika.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://liverguac-my.sharepoint.com/personal/a_siyambalapitiyage_rgu_ac_uk/Documents/Desktop/DSGP/DSGP_Group_38/WholeSale-Price-Model/data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="83" documentId="8_{DBDE29C9-DF6E-4BC9-ABC1-633918917E58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1DBDB6B0-B88A-4BE7-919C-DECE394FEF83}"/>
+  <xr:revisionPtr revIDLastSave="105" documentId="8_{DBDE29C9-DF6E-4BC9-ABC1-633918917E58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9C2AD3A4-95AE-47A7-8FF8-8E8C8DA14376}"/>
   <bookViews>
-    <workbookView xWindow="3552" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{215EF489-9573-4990-96B9-A28CAE1C2861}"/>
+    <workbookView xWindow="11712" yWindow="0" windowWidth="11424" windowHeight="12336" xr2:uid="{215EF489-9573-4990-96B9-A28CAE1C2861}"/>
   </bookViews>
   <sheets>
     <sheet name="Wholesale" sheetId="2" r:id="rId1"/>
@@ -1439,7 +1439,10 @@
     <col min="8" max="8" width="10.109375" style="3" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="8.5546875" style="3" bestFit="1" customWidth="1"/>
     <col min="10" max="11" width="9.21875" style="3" bestFit="1" customWidth="1"/>
-    <col min="12" max="56" width="8.5546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.5546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9.44140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.77734375" style="3" bestFit="1" customWidth="1"/>
+    <col min="15" max="56" width="8.5546875" style="3" bestFit="1" customWidth="1"/>
     <col min="57" max="16384" width="8.88671875" style="3"/>
   </cols>
   <sheetData>
@@ -16983,9 +16986,15 @@
       <c r="K98" s="9">
         <v>235</v>
       </c>
-      <c r="L98" s="9"/>
-      <c r="M98" s="8"/>
-      <c r="N98" s="8"/>
+      <c r="L98" s="9">
+        <v>296</v>
+      </c>
+      <c r="M98" s="9">
+        <v>275</v>
+      </c>
+      <c r="N98" s="9">
+        <v>260</v>
+      </c>
       <c r="O98" s="8"/>
       <c r="P98" s="8"/>
       <c r="Q98" s="8"/>
@@ -17061,9 +17070,15 @@
       <c r="K99" s="9">
         <v>105</v>
       </c>
-      <c r="L99" s="9"/>
-      <c r="M99" s="6"/>
-      <c r="N99" s="8"/>
+      <c r="L99" s="9">
+        <v>170</v>
+      </c>
+      <c r="M99" s="6">
+        <v>110</v>
+      </c>
+      <c r="N99" s="9">
+        <v>125</v>
+      </c>
       <c r="O99" s="8"/>
       <c r="P99" s="8"/>
       <c r="Q99" s="8"/>
@@ -17139,9 +17154,15 @@
       <c r="K100" s="6">
         <v>125</v>
       </c>
-      <c r="L100" s="6"/>
-      <c r="M100" s="6"/>
-      <c r="N100" s="6"/>
+      <c r="L100" s="6">
+        <v>207</v>
+      </c>
+      <c r="M100" s="6">
+        <v>75</v>
+      </c>
+      <c r="N100" s="6">
+        <v>45</v>
+      </c>
       <c r="O100" s="6"/>
       <c r="P100" s="6"/>
       <c r="Q100" s="6"/>
@@ -17217,9 +17238,15 @@
       <c r="K101" s="6">
         <v>135</v>
       </c>
-      <c r="L101" s="6"/>
-      <c r="M101" s="6"/>
-      <c r="N101" s="6"/>
+      <c r="L101" s="6">
+        <v>167</v>
+      </c>
+      <c r="M101" s="6">
+        <v>135</v>
+      </c>
+      <c r="N101" s="6">
+        <v>290</v>
+      </c>
       <c r="O101" s="6"/>
       <c r="P101" s="6"/>
       <c r="Q101" s="6"/>
@@ -17295,9 +17322,15 @@
       <c r="K102" s="6">
         <v>105</v>
       </c>
-      <c r="L102" s="6"/>
-      <c r="M102" s="6"/>
-      <c r="N102" s="6"/>
+      <c r="L102" s="6">
+        <v>90</v>
+      </c>
+      <c r="M102" s="6">
+        <v>95</v>
+      </c>
+      <c r="N102" s="6">
+        <v>110</v>
+      </c>
       <c r="O102" s="6"/>
       <c r="P102" s="6"/>
       <c r="Q102" s="6"/>
@@ -17373,9 +17406,15 @@
       <c r="K103" s="6">
         <v>290</v>
       </c>
-      <c r="L103" s="6"/>
-      <c r="M103" s="6"/>
-      <c r="N103" s="6"/>
+      <c r="L103" s="6">
+        <v>375</v>
+      </c>
+      <c r="M103" s="6">
+        <v>250</v>
+      </c>
+      <c r="N103" s="6">
+        <v>195</v>
+      </c>
       <c r="O103" s="6"/>
       <c r="P103" s="6"/>
       <c r="Q103" s="6"/>

</xml_diff>